<commit_message>
Rewrite brand-mention replies to read as natural feedback
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015dXgfxu1ugCxsD9bCGxkqs
</commit_message>
<xml_diff>
--- a/lynkk-reddit-leads/results/2026-10-11/campaign_replies_2026-10-11.xlsx
+++ b/lynkk-reddit-leads/results/2026-10-11/campaign_replies_2026-10-11.xlsx
@@ -526,12 +526,12 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>1 lead (looking for a tool)</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n">
+      <c r="B2" t="n">
         <v>1</v>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -544,30 +544,30 @@
           <t>https://www.reddit.com/r/AIAssisted/comments/1wq1m2t/which_ai_meeting_note_taker_are_you_using/</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>post</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>r/AIAssisted</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>u/Rist0o0</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Which AI meeting note taker are you using?</t>
         </is>
       </c>
-      <c r="I2" s="2" t="n">
+      <c r="I2" t="n">
         <v>84</v>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>high_purchase_intent</t>
         </is>
@@ -584,11 +584,11 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>If your in-person meetings happen where a laptop is open, you may not need a separate recorder; a laptop mic is fine for a small room, and having everything in one place matters more than people expect. A recorder makes sense for site visits or coffee meetings.
-I work on Lynkk, so I'm biased, but it covers both from one account: the Mac app or Chrome extension records online calls without a bot joining, and in person you can record from the laptop mic in the browser. Each meeting gets a brief with decisions and action items, and the timestamps play the recording from that moment. It's Mac and web only, no phone app.</t>
-        </is>
-      </c>
-      <c r="N2" s="2" t="inlineStr">
+          <t>Depends a lot on where your in-person meetings happen. If there's usually a laptop on the table anyway, I'd try recording from that before buying a Plaud or Pocket. A laptop mic is fine for a small room, and you end up with everything in one app instead of two, which you'll appreciate when you're looking for something from three weeks ago. A recorder makes more sense if you're often in cafes or on site.
+Full disclosure, I work on Lynkk, which does that combo (calls without a bot, in-person from the browser), so I'm biased. But the one-place thing matters whichever tool you pick.</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
         <is>
           <t>If you want to try it, there's a free plan at lynkk.ai.</t>
         </is>
@@ -600,12 +600,12 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>1 lead (looking for a tool)</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n">
+      <c r="B3" t="n">
         <v>2</v>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -618,17 +618,17 @@
           <t>https://www.reddit.com/r/PLAUDAI/comments/1x1tha4/lawyers_using_plaud_or_other_ai_notetakers_for/</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>post</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>r/PLAUDAI</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>u/Party_History2839</t>
         </is>
@@ -638,10 +638,10 @@
           <t>Lawyers using Plaud or other AI note-takers for client consultations — what has your experience been?</t>
         </is>
       </c>
-      <c r="I3" s="2" t="n">
+      <c r="I3" t="n">
         <v>82</v>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>comparison</t>
         </is>
@@ -658,11 +658,12 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>For in-person consults, a cheap USB boundary mic on the table helps accuracy more than switching apps. For the weeks-later problem, judge tools on whether the summary keeps decisions and open questions with timestamps back to the recording, so you can check exact wording before drafting.
-I work on Lynkk, so take this with that in mind. It records in-person meetings from the laptop mic in the browser and video calls through the Mac app with no bot joining. Each note gets a brief with decisions, open questions and action items, and every timestamp plays the recording from that moment. We never train on your conversations, but put your confidentiality questions to any vendor in writing, us included.</t>
-        </is>
-      </c>
-      <c r="N3" s="2" t="inlineStr">
+          <t>The weeks-later gap is the real test, and most demos never show it. Record a consult, don't touch it for two weeks, then try to draft from the notes alone and see what's missing. Day-one summaries all look fine.
+Also +1 on a cheap boundary mic for in-person, it matters more than the app.
+I'm on the Lynkk team, so grain of salt, but if you want a software-only option to compare against Plaud Desktop, it records in the browser for in-person and through a Mac app for calls, and every point in the notes links back to the spot in the recording. Worth running the same consult through both.</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
         <is>
           <t>If you want to try it, there's a free plan at lynkk.ai.</t>
         </is>
@@ -674,12 +675,12 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>1 lead (looking for a tool)</t>
         </is>
       </c>
-      <c r="B4" s="2" t="n">
+      <c r="B4" t="n">
         <v>3</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -692,17 +693,17 @@
           <t>https://www.reddit.com/r/AiNoteTaker/comments/1wzy65s/any_ai_tool_that_can_handle_both_online_and/</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>post</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>r/AiNoteTaker</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>u/jordanconnelly</t>
         </is>
@@ -712,10 +713,10 @@
           <t>Any AI tool that can handle both online and offline meeting notes?</t>
         </is>
       </c>
-      <c r="I4" s="2" t="n">
+      <c r="I4" t="n">
         <v>80</v>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>high_purchase_intent</t>
         </is>
@@ -732,11 +733,11 @@
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>Choose by where everything ends up, not how it records; one searchable library is what stops the digging.
-I work on Lynkk, so I'm biased. It handles two of your three: the Mac app notices Zoom, Meet, Teams, FaceTime and WhatsApp calls and records without a bot, and in-person meetings can be recorded from the laptop mic in the browser. Everything lands in one place, and you can ask questions across your notes by person, company or project. Honest gap: there's no phone app, so native iPhone calls aren't covered. Taking important calls through FaceTime or WhatsApp on the Mac gets them in too.</t>
-        </is>
-      </c>
-      <c r="N4" s="2" t="inlineStr">
+          <t>Phone calls are the annoying one. Almost nothing can record a regular iPhone call, so people either take important calls on the laptop (FaceTime or WhatsApp desktop) or live with a separate app for those.
+Zoom plus in-person in one place is the easy part. Disclosure, I work on Lynkk, which handles those two and keeps them searchable together, but there's no phone app, so it wouldn't fix the iPhone bit. Whatever you go with, I'd rank 'one place to search' above anything else on the feature list.</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
         <is>
           <t>If you want to try it, there's a free plan at lynkk.ai.</t>
         </is>
@@ -748,12 +749,12 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>1 lead (looking for a tool)</t>
         </is>
       </c>
-      <c r="B5" s="2" t="n">
+      <c r="B5" t="n">
         <v>4</v>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -766,17 +767,17 @@
           <t>https://www.reddit.com/r/AiNoteTaker/comments/1wm4zsu/can_any_ai_notetaker_show_how_a_decision_changed/</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>post</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>r/AiNoteTaker</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>u/FinishTough23</t>
         </is>
@@ -786,10 +787,10 @@
           <t>Can any AI notetaker show how a decision changed across multiple meetings?</t>
         </is>
       </c>
-      <c r="I5" s="2" t="n">
+      <c r="I5" t="n">
         <v>76</v>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>tool_recommendation</t>
         </is>
@@ -806,11 +807,11 @@
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>I haven't seen anything that builds a clean decision changelog automatically, so it's a combination: summaries that keep decisions apart from concerns, questions asked across all of a project's meetings, and saying changes out loud on the call ('we're moving launch to November because of lead times').
-I work on Lynkk, so I'm biased. Its chat answers only from your own notes, can find notes by project, and lists decisions with citation chips that open the note at the exact moment, so you can click through each step and confirm a suggestion actually became an agreement. It's not a dedicated timeline view, but it covers the 'what's current and why' question.</t>
-        </is>
-      </c>
-      <c r="N5" s="2" t="inlineStr">
+          <t>This is the thing summaries are worst at, because each one only knows its own meeting. What tends to work better is asking across the whole project ('what's the current launch date and when did it change?') and only trusting answers that point to the specific meeting and moment, so you can click through and see whether it was a real decision or just someone floating it.
+Disclosure, I work on Lynkk, and that's roughly how its chat works: answers from your own notes, with citations you can click. Not a proper decision timeline though. Would love to see someone build that.</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
         <is>
           <t>If you want to try it, there's a free plan at lynkk.ai.</t>
         </is>
@@ -822,12 +823,12 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>1 lead (looking for a tool)</t>
         </is>
       </c>
-      <c r="B6" s="2" t="n">
+      <c r="B6" t="n">
         <v>5</v>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -840,17 +841,17 @@
           <t>https://www.reddit.com/r/softwaresworthpaying/comments/1wzp2i0/do_we_need_another_ai_meeting_note_taker_for/</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>post</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>r/softwaresworthpaying</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>u/BakerInfamous6110</t>
         </is>
@@ -860,10 +861,10 @@
           <t>Do we need another AI meeting note taker for microsoft teams if we have Copilot?</t>
         </is>
       </c>
-      <c r="I6" s="2" t="n">
+      <c r="I6" t="n">
         <v>74</v>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>comparison</t>
         </is>
@@ -880,11 +881,11 @@
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>Copilot covers meetings your tenant hosts, so customer links are the gap. For finance, count last month's important customer calls outside Teams; that number is the case. Keep Copilot for internal meetings and only add seats for people on external calls.
-I work on Lynkk, so I'm biased. The Mac app notices calls in Zoom, Google Meet, Teams, Slack huddles and Webex and records from the laptop with no bot, so it doesn't matter whose link it is. There's also a bot that can join Zoom, Meet and Teams links if you prefer. Caveat: the Mac app needs Apple silicon.</t>
-        </is>
-      </c>
-      <c r="N6" s="2" t="inlineStr">
+          <t>Copilot's fine for internal stuff, but it really only covers meetings your tenant hosts, so customer calls on their Zoom links fall through. For the budget conversation I'd count how many important customer calls last month were outside Teams. That number usually settles it.
+If you do add something, look for one that records from the laptop instead of joining as a bot, then it doesn't matter whose link it is. (I work on Lynkk, which works that way on Mac, so yes, biased. Apple silicon only though.)</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
         <is>
           <t>If you want to try it, there's a free plan at lynkk.ai.</t>
         </is>
@@ -896,12 +897,12 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>1 lead (looking for a tool)</t>
         </is>
       </c>
-      <c r="B7" s="2" t="n">
+      <c r="B7" t="n">
         <v>6</v>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -914,30 +915,30 @@
           <t>https://www.reddit.com/r/sales/comments/1wk7yt9/tablet_apps_and_ai_tools/</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>post</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>r/sales</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>u/throwaway09251975</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>Tablet, Apps, and AI Tools</t>
         </is>
       </c>
-      <c r="I7" s="2" t="n">
+      <c r="I7" t="n">
         <v>72</v>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>high_purchase_intent</t>
         </is>
@@ -954,11 +955,11 @@
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>Since customers are fine with recording, record instead of converting handwriting; you get a summary with next steps you didn't have to write, which maps straight onto a follow-up email.
-I work on Lynkk, so I'm biased. You can record an in-person meeting from a laptop mic in the browser and get a brief with decisions, action items with owners and due dates, and open questions. Honest limits: there's no tablet or phone app, and it doesn't sync to Salesforce, so the CRM step stays manual. If you're on a laptop in meetings anyway, it covers the notes and next steps part.</t>
-        </is>
-      </c>
-      <c r="N7" s="2" t="inlineStr">
+          <t>If customers are fine with recording, I'd skip the tablet and handwriting route. You'd still be summarizing your own notes afterwards. Record the meeting, let the tool pull the next steps, and the follow-up email is mostly done.
+Salesforce is where most of these tools get vague, so ask straight out whether it updates fields or just hands you text. Disclosure: I work on Lynkk, which covers the record and next steps part from a laptop, but it doesn't sync to Salesforce, so that bit would stay manual.</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
         <is>
           <t>If you want to try it, there's a free plan at lynkk.ai.</t>
         </is>
@@ -970,12 +971,12 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>1 lead (looking for a tool)</t>
         </is>
       </c>
-      <c r="B8" s="2" t="n">
+      <c r="B8" t="n">
         <v>7</v>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -988,30 +989,30 @@
           <t>https://www.reddit.com/r/PlaudNoteUsers/comments/1x12i9y/what_ai_note_taking_apps_are_you_using_for/</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>post</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>r/PlaudNoteUsers</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>u/QuietlyKevin07</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>What AI note taking apps are you using for meetings?</t>
         </is>
       </c>
-      <c r="I8" s="2" t="n">
+      <c r="I8" t="n">
         <v>72</v>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>tool_recommendation</t>
         </is>
@@ -1028,11 +1029,11 @@
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>For small details, what matters is whether the summary links back to the exact moment in the recording, and whether you can search across all meetings. Test with a real 60 to 90 minute call; that's where summaries get vague.
-I work on Lynkk, so I'm biased. Every takeaway in its brief has a timestamp that plays the recording from that moment, and you can ask questions across your notes and get answers with citations back to the moment. Recordings go up to 2 hours each. It's Mac, Chrome and web rather than a hardware recorder, so it suits calls and laptop-in-the-room meetings.</t>
-        </is>
-      </c>
-      <c r="N8" s="2" t="inlineStr">
+          <t>The biggest difference on long meetings is whether you can jump from a line in the summary straight to that moment in the audio. Saves so much scrubbing. And test with a real 90 minute meeting, not a 10 minute demo; that's where summaries start getting mushy.
+(Disclosure: I work on Lynkk, which does the timestamp-to-audio thing, but it's Mac, Chrome and web, not a pocket recorder, so it's a different setup from Plaud.)</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
         <is>
           <t>If you want to try it, there's a free plan at lynkk.ai.</t>
         </is>
@@ -1044,12 +1045,12 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>1 lead (looking for a tool)</t>
         </is>
       </c>
-      <c r="B9" s="2" t="n">
+      <c r="B9" t="n">
         <v>8</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -1062,17 +1063,17 @@
           <t>https://www.reddit.com/r/AgentsOfAI/comments/1wtfbyj/one_ai_meeting_note_taker_for_microsoft_teams_and/</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>post</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>r/AgentsOfAI</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>u/Then_Date1452</t>
         </is>
@@ -1082,10 +1083,10 @@
           <t>One AI meeting note taker for Microsoft Teams and all the zoom links?</t>
         </is>
       </c>
-      <c r="I9" s="2" t="n">
+      <c r="I9" t="n">
         <v>72</v>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>comparison</t>
         </is>
@@ -1102,11 +1103,11 @@
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>Pilot it on the external calls first. Watch for customers' Zoom settings holding bots in the waiting room, recordings landing in different places depending on host, and retention differing between personal and company accounts.
-I work on Lynkk, so I'm biased. It does both platforms from one archive: a bot that joins Teams, Zoom and Meet links (or auto-joins from the calendar), plus a Mac app and Chrome extension that record without a bot when a bot gets blocked. A workspace gives everyone Pro and keeps the record with the company. Limit: workspaces are up to 10 seats, so it fits a small team, not a big rollout.</t>
-        </is>
-      </c>
-      <c r="N9" s="2" t="inlineStr">
+          <t>The thing that breaks in practice is external Zoom calls where the host's settings hold bots in the waiting room. So whatever you pick, make sure it can also record from the user's own machine as a fallback. Then run a two-week pilot with whoever lives on Zoom and just count how many external calls actually got captured.
+I'm on the Lynkk team, bias noted. It has a bot for Teams, Zoom and Meet plus a no-bot Mac app and Chrome extension for the blocked cases, all in one archive. Workspaces cap at 10 seats though, so only relevant if this client's team is small.</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
         <is>
           <t>If you want to try it, there's a free plan at lynkk.ai.</t>
         </is>
@@ -1118,12 +1119,12 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>1 lead (looking for a tool)</t>
         </is>
       </c>
-      <c r="B10" s="2" t="n">
+      <c r="B10" t="n">
         <v>9</v>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -1136,35 +1137,35 @@
           <t>https://www.reddit.com/r/AIAssisted/comments/1wj0zra/what_ai_meeting_note_taker_are_you_actually_using/</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>post</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>r/AIAssisted</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>u/jimmybobjoeflow</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>What AI meeting note taker are you actually using?</t>
         </is>
       </c>
-      <c r="I10" s="2" t="n">
+      <c r="I10" t="n">
         <v>70</v>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>tool_recommendation</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>Good lead. Asks which note taker people use.</t>
         </is>
@@ -1176,11 +1177,11 @@
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>Some review is still worth it, but it can be a two-minute skim if decisions, action items and open questions are separate lists with timestamps back to the recording. Saying owners and deadlines out loud at the end of the call helps a lot too.
-I work on Lynkk, so I'm biased. Its meeting brief lists decisions with context, action items with owner, due date and priority, and open questions, and every timestamp plays the recording from that moment, so checking an item takes seconds. It records Zoom, Meet and Teams without a bot from the Mac app or Chrome extension.</t>
-        </is>
-      </c>
-      <c r="N10" s="2" t="inlineStr">
+          <t>You'll probably always do some review, but it can be a two-minute skim instead of a reread. What cuts it down most is when every action item has a timestamp you can click to hear the original moment, so you only check the ones that look off. Saying owners and dates out loud at the end of the call helps a ton too.
+Disclosure, I work on Lynkk, which is built around that click-to-check idea. Honestly though, the verbal recap at the end helps with any tool.</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
         <is>
           <t>If you want to try it, there's a free plan at lynkk.ai.</t>
         </is>
@@ -1192,12 +1193,12 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>1 lead (looking for a tool)</t>
         </is>
       </c>
-      <c r="B11" s="2" t="n">
+      <c r="B11" t="n">
         <v>10</v>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -1210,17 +1211,17 @@
           <t>https://www.reddit.com/r/AI_Agents/comments/1wq1vrs/any_fathom_ai_alternatives_that_work_better_with/</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>post</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>r/AI_Agents</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>u/Sash19</t>
         </is>
@@ -1230,10 +1231,10 @@
           <t>Any Fathom AI alternatives that work better with agent workflows?</t>
         </is>
       </c>
-      <c r="I11" s="2" t="n">
+      <c r="I11" t="n">
         <v>66</v>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>comparison</t>
         </is>
@@ -1250,11 +1251,11 @@
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>Two setups work: pipe transcripts into your agent (flexible, but the agent does the retrieval), or ask questions inside the notes tool if it searches across meetings and cites sources. For follow-ups and old decisions, the second is often enough.
-I work on Lynkk, so I'm biased. Its chat answers only from your own notes, finds them by person, company or project, lists open tasks and decisions with citations to the moment, and can take actions behind a confirm step, like creating a Jira issue or a calendar event. You can also ask it from Slack. It's a different shape from MCP, so it depends on whether you need your own agent in the loop.</t>
-        </is>
-      </c>
-      <c r="N11" s="2" t="inlineStr">
+          <t>Depends whether you need the meeting data inside your own agent or just need answers. If it's mostly 'what did we decide with X' and 'what's still open', asking inside the notes tool is simpler than wiring transcripts into an agent. If the agent needs to act on it alongside other context, then yeah, your MCP route makes sense.
+I work on Lynkk so I'm biased, but it's the first kind: you ask across your notes, get answers that link back to the moment, and can create a Jira issue from there. Not sure it fits if you need it inside your own agent.</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
         <is>
           <t>If you want to try it, there's a free plan at lynkk.ai.</t>
         </is>
@@ -1266,12 +1267,12 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>1 lead (looking for a tool)</t>
         </is>
       </c>
-      <c r="B12" s="2" t="n">
+      <c r="B12" t="n">
         <v>11</v>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -1284,17 +1285,17 @@
           <t>https://www.reddit.com/r/AIWorkStack/comments/1x14cj5/are_ai_notetaking_tools_actually_better_than/</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>post</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>r/AIWorkStack</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>u/lebron7</t>
         </is>
@@ -1304,15 +1305,15 @@
           <t>Are AI note-taking tools actually better than taking notes yourself?</t>
         </is>
       </c>
-      <c r="I12" s="2" t="n">
+      <c r="I12" t="n">
         <v>66</v>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>tool_recommendation</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>Disclosed vendor replies already appear in this thread.</t>
         </is>
@@ -1324,11 +1325,11 @@
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>Checking is the right instinct; the trick is making it fast. Timestamps on each takeaway that play the original moment turn verification into a ten-second job, and saying decisions and owners out loud at the end of the call makes summaries much more reliable.
-I work on Lynkk, so I'm biased. That's how its meeting brief works: every takeaway and action item has a timestamp that plays the recording from that moment, and you can search or ask questions across all your notes afterward. It records without a bot from the Mac app or Chrome extension, and in person from the browser.</t>
-        </is>
-      </c>
-      <c r="N12" s="2" t="inlineStr">
+          <t>Checking is the right call. What makes it workable is being able to click a line in the summary and hear the original moment, so checking a detail takes seconds instead of rereading the transcript. Small details are exactly where summaries slip, so I'd trust the summary for the gist and the recording for names and numbers.
+(I work on Lynkk, so bias disclosed. It does the click-to-hear thing, plus search across all your meetings afterwards.)</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
         <is>
           <t>If you want to try it, there's a free plan at lynkk.ai.</t>
         </is>
@@ -1340,12 +1341,12 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>1 lead (looking for a tool)</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
+      <c r="B13" t="n">
         <v>12</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -1358,17 +1359,17 @@
           <t>https://www.reddit.com/r/MyAIAssistant/comments/1wjsca7/my_ai_summarized_a_meeting_and_invented_an_action/</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>post</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>r/MyAIAssistant</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>u/Morphius007</t>
         </is>
@@ -1378,10 +1379,10 @@
           <t>My AI summarized a meeting and invented an action item that committed us to a go-live date.</t>
         </is>
       </c>
-      <c r="I13" s="2" t="n">
+      <c r="I13" t="n">
         <v>66</v>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>problem_seeking_solution</t>
         </is>
@@ -1398,11 +1399,11 @@
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>The reliable fix is evidence: every action item should link to the moment it came from, and anything without a source stays a draft. Have owners confirm their own items, and end calls with a 60-second recap of owners and dates said out loud.
-I work on Lynkk, so I'm biased. Its brief keeps decisions, action items and open questions separate, and every item has a timestamp that plays the recording from that moment, so an invented 'Ship Phase 2 by Friday' is quick to catch because there's nothing to click back to. Sending items to Jira is a manual step, so nothing hits the board without a person.</t>
-        </is>
-      </c>
-      <c r="N13" s="2" t="inlineStr">
+          <t>That 'inferred urgency' thing is exactly why action items need a source. Simplest rule: every action item links to the moment it was said, and anything without a source stays a draft. That catches invented deadlines in seconds. Also have owners confirm their own items instead of the PM approving everything.
+Disclosure, I work on Lynkk. Its action items each carry a timestamp back to the recording, and nothing goes to Jira unless someone sends it by hand.</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
         <is>
           <t>If you want to try it, there's a free plan at lynkk.ai.</t>
         </is>
@@ -1414,12 +1415,12 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>1 lead (looking for a tool)</t>
         </is>
       </c>
-      <c r="B14" s="2" t="n">
+      <c r="B14" t="n">
         <v>13</v>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -1432,17 +1433,17 @@
           <t>https://www.reddit.com/r/PLAUDAI/comments/1x1tha4/lawyers_using_plaud_or_other_ai_notetakers_for/</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>comment</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>r/PLAUDAI</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>u/Party_History2839</t>
         </is>
@@ -1452,10 +1453,10 @@
           <t>Lawyers using Plaud or other AI note-takers for client consultations — what has your experience been?</t>
         </is>
       </c>
-      <c r="I14" s="2" t="n">
+      <c r="I14" t="n">
         <v>60</v>
       </c>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>comparison</t>
         </is>
@@ -1472,11 +1473,10 @@
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>Reasonable worry. Whatever you pick, export regularly so you're never locked in, and pilot two tools on real consultations before committing firm-wide.
-I work on Lynkk, so I'm biased, but if you want a second tool to compare: it records consultations from the laptop mic in the browser and video calls through the Mac app without a bot, and gives a brief with decisions and open questions that link back to the recording. It's software only, so no hardware to commit to.</t>
-        </is>
-      </c>
-      <c r="N14" s="2" t="inlineStr">
+          <t>Totally fair worry. Whatever you pick, export your recordings regularly so you're never stuck, and do a short side-by-side with a second tool before recommending anything firm-wide. (I work on Lynkk, so I'm one of the options. It's software only, so there's no hardware to bet on.)</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
         <is>
           <t>If you want to try it, there's a free plan at lynkk.ai.</t>
         </is>
@@ -1488,12 +1488,12 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>1 lead (looking for a tool)</t>
         </is>
       </c>
-      <c r="B15" s="2" t="n">
+      <c r="B15" t="n">
         <v>14</v>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -1506,30 +1506,30 @@
           <t>https://www.reddit.com/r/AIToolTalks/comments/1ws9lds/which_ai_meeting_note_taker_are_you_using/</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>post</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>r/AIToolTalks</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>u/Rist0o0</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>Which AI meeting note taker are you using?</t>
         </is>
       </c>
-      <c r="I15" s="2" t="n">
+      <c r="I15" t="n">
         <v>60</v>
       </c>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>tool_recommendation</t>
         </is>
@@ -1546,11 +1546,10 @@
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>Depends on your mix, but keeping online and in-person meetings in one searchable place matters most.
-I work on Lynkk, so I'm biased. It records online calls without a bot from the Mac app or Chrome extension, records in-person meetings from the laptop mic in the browser, and gives each meeting a brief with decisions and action items linked back to the recording.</t>
-        </is>
-      </c>
-      <c r="N15" s="2" t="inlineStr">
+          <t>Mostly depends on whether you have in-person meetings too. If you do, keep everything in one tool, otherwise you end up searching two places later. I'm on the Lynkk team, which does calls without a bot plus in-person from the browser, but I'd give the same advice for any tool.</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
         <is>
           <t>If you want to try it, there's a free plan at lynkk.ai.</t>
         </is>
@@ -1562,12 +1561,12 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" t="inlineStr">
         <is>
           <t>1 lead (looking for a tool)</t>
         </is>
       </c>
-      <c r="B16" s="2" t="n">
+      <c r="B16" t="n">
         <v>15</v>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -1580,17 +1579,17 @@
           <t>https://www.reddit.com/r/MyAIAssistant/comments/1wli9fz/my_meetingnotes_ai_invented_action_owners_who/</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>post</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>r/MyAIAssistant</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>u/Morphius007</t>
         </is>
@@ -1600,10 +1599,10 @@
           <t>My meeting-notes AI invented action owners who were not even in the meeting.</t>
         </is>
       </c>
-      <c r="I16" s="2" t="n">
+      <c r="I16" t="n">
         <v>58</v>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="J16" t="inlineStr">
         <is>
           <t>problem_seeking_solution</t>
         </is>
@@ -1620,11 +1619,10 @@
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>The stronger check than attendee lists is evidence: an owner should only be set when someone said it, with a link to that moment; otherwise it's 'owner needed'. A verbal recap of owners at the end of the call removes most of the guessing.
-I work on Lynkk, so I'm biased. Its action items carry owner, due date and priority, each with a timestamp that plays the recording from that moment, so you can check whether an owner was actually named before anything is sent on.</t>
-        </is>
-      </c>
-      <c r="N16" s="2" t="inlineStr">
+          <t>Attendee-only is a good guardrail, but I'd go one step further: only set an owner when someone actually said it, with a link to that moment. Otherwise mark it 'owner needed'. A 30-second recap at the end ('Priya has the roadmap, Friday') removes most of the guessing. (Disclosure: I work on Lynkk, where every action item links back to the recording, which makes checking this pretty quick.)</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
         <is>
           <t>If you want to try it, there's a free plan at lynkk.ai.</t>
         </is>
@@ -1636,12 +1634,12 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" t="inlineStr">
         <is>
           <t>1 lead (looking for a tool)</t>
         </is>
       </c>
-      <c r="B17" s="2" t="n">
+      <c r="B17" t="n">
         <v>16</v>
       </c>
       <c r="C17" s="3" t="inlineStr">
@@ -1654,17 +1652,17 @@
           <t>https://www.reddit.com/r/PLAUDAI/comments/1x1tha4/lawyers_using_plaud_or_other_ai_notetakers_for/</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>comment</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>r/PLAUDAI</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>u/Party_History2839</t>
         </is>
@@ -1674,10 +1672,10 @@
           <t>Lawyers using Plaud or other AI note-takers for client consultations — what has your experience been?</t>
         </is>
       </c>
-      <c r="I17" s="2" t="n">
+      <c r="I17" t="n">
         <v>55</v>
       </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="J17" t="inlineStr">
         <is>
           <t>comparison</t>
         </is>
@@ -1694,11 +1692,10 @@
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>Fair reason to look around: if you need recording, transcription and a reliable summary, focus beats agent features. Test any alternative against your top three needs on a real consultation.
-I work on Lynkk, so I'm biased, but that's the core of what it does: record (browser for in-person, Mac app for calls, no bot), transcribe, and give a brief with decisions, open questions and action items that link back to the recording.</t>
-        </is>
-      </c>
-      <c r="N17" s="2" t="inlineStr">
+          <t>Makes sense. If what you need is record, transcribe and summarize reliably, the agent features are just noise. I'd write down the three things you actually rely on and test alternatives against only those. (Biased, I work on Lynkk, which sticks to that core: recording, transcript, and a brief that links back to the audio.)</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
         <is>
           <t>If you want to try it, there's a free plan at lynkk.ai.</t>
         </is>
@@ -1710,12 +1707,12 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="A18" t="inlineStr">
         <is>
           <t>1 lead (looking for a tool)</t>
         </is>
       </c>
-      <c r="B18" s="2" t="n">
+      <c r="B18" t="n">
         <v>17</v>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -1728,17 +1725,17 @@
           <t>https://www.reddit.com/r/PLAUDAI/comments/1x1tha4/lawyers_using_plaud_or_other_ai_notetakers_for/</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>comment</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>r/PLAUDAI</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>u/Overall_Fold7937</t>
         </is>
@@ -1748,10 +1745,10 @@
           <t>Lawyers using Plaud or other AI note-takers for client consultations — what has your experience been?</t>
         </is>
       </c>
-      <c r="I18" s="2" t="n">
+      <c r="I18" t="n">
         <v>55</v>
       </c>
-      <c r="J18" s="2" t="inlineStr">
+      <c r="J18" t="inlineStr">
         <is>
           <t>workflow_problem</t>
         </is>
@@ -1768,11 +1765,10 @@
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>Mixed-language meetings are hard for most engines. Setting the languages up front and adding custom words for names helps, and a short hand-checked sample tells you if it's the audio or the model.
-I work on Lynkk, so I'm biased. It transcribes 17 languages with auto-detect (four of them in beta) and has a custom words dictionary, so it might be worth a side-by-side test on one of your mixed meetings.</t>
-        </is>
-      </c>
-      <c r="N18" s="2" t="inlineStr">
+          <t>Mixed language is rough for most engines. Setting the languages explicitly, if your tool lets you, and adding names and terms to a custom vocab usually helps more than anything. If you want a comparison point, I work on Lynkk, which does 17 languages with auto-detect plus a custom words list. Might be worth one side-by-side on a mixed meeting.</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
         <is>
           <t>If you want to try it, there's a free plan at lynkk.ai.</t>
         </is>
@@ -1784,12 +1780,12 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" t="inlineStr">
         <is>
           <t>1 lead (looking for a tool)</t>
         </is>
       </c>
-      <c r="B19" s="2" t="n">
+      <c r="B19" t="n">
         <v>18</v>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -1802,17 +1798,17 @@
           <t>https://www.reddit.com/r/negotiation/comments/1x1qct6/is_there_an_ai_tool_that_can_tell_me_exactly/</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>post</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>r/negotiation</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>u/belligerent_vogue</t>
         </is>
@@ -1822,10 +1818,10 @@
           <t>Is there an AI tool that can tell me exactly where a sales negotiation went wrong?</t>
         </is>
       </c>
-      <c r="I19" s="2" t="n">
+      <c r="I19" t="n">
         <v>52</v>
       </c>
-      <c r="J19" s="2" t="inlineStr">
+      <c r="J19" t="inlineStr">
         <is>
           <t>problem_seeking_solution</t>
         </is>
@@ -1842,11 +1838,10 @@
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>Start with five lost and five won deals, and review only the stretch from first price mention onward; patterns show up fast across ten calls.
-I work on Lynkk, so I'm biased, and it isn't a coaching tool. But its Sales Call summary and timestamped takeaways let you jump to the price discussion instead of replaying an hour, and you can ask questions across calls with answers that cite the moment. It may help with the review time, not the scoring.</t>
-        </is>
-      </c>
-      <c r="N19" s="2" t="inlineStr">
+          <t>I'd start smaller than a coaching platform. Take five lost deals and five won ones and only listen from the first price mention onward. Patterns show up faster than you'd think. (I work on Lynkk. It's not a coaching tool, but its timestamps let you jump straight to the price discussion instead of replaying the whole hour, which might at least cut the review time.)</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
         <is>
           <t>If you want to try it, there's a free plan at lynkk.ai.</t>
         </is>
@@ -1858,12 +1853,12 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="A20" t="inlineStr">
         <is>
           <t>1 lead (looking for a tool)</t>
         </is>
       </c>
-      <c r="B20" s="2" t="n">
+      <c r="B20" t="n">
         <v>19</v>
       </c>
       <c r="C20" s="3" t="inlineStr">
@@ -1876,30 +1871,30 @@
           <t>https://www.reddit.com/r/AIDiscussion/comments/1wymbzg/is_an_ai_meeting_assistant_saving_you_work_after/</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>post</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>r/AIDiscussion</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>u/Doug19</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="H20" t="inlineStr">
         <is>
           <t>Is an AI meeting assistant saving you work after the call?</t>
         </is>
       </c>
-      <c r="I20" s="2" t="n">
+      <c r="I20" t="n">
         <v>52</v>
       </c>
-      <c r="J20" s="2" t="inlineStr">
+      <c r="J20" t="inlineStr">
         <is>
           <t>general_discussion</t>
         </is>
@@ -1916,11 +1911,10 @@
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>The useful part is structure, not the summary: decisions, action items with owners, and open questions as separate lists, each linked to the moment it came from. 'We could try this' belongs in open questions.
-I work on Lynkk, so I'm biased. Its brief is built that way, with timestamps that play the recording, and without a bot from the Mac app or Chrome extension, which sounds like what you liked about Bluedot.</t>
-        </is>
-      </c>
-      <c r="N20" s="2" t="inlineStr">
+          <t>The summary itself rarely saves time. What helps is when 'we could try this' gets filed as an open question instead of a decision, and you can click back to hear how it was actually said. (Disclosure: I work on Lynkk, which records without a bot too. Curious what other people find actually gets opened after the meeting.)</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
         <is>
           <t>If you want to try it, there's a free plan at lynkk.ai.</t>
         </is>
@@ -1932,12 +1926,12 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" t="inlineStr">
         <is>
           <t>2 engagement (discussion)</t>
         </is>
       </c>
-      <c r="B21" s="2" t="n">
+      <c r="B21" t="n">
         <v>20</v>
       </c>
       <c r="C21" s="3" t="inlineStr">
@@ -1950,17 +1944,17 @@
           <t>https://www.reddit.com/r/ProductivityApps/comments/1x1hlb5/anyone_automated_turning_meeting_notes_into/</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>post</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>r/ProductivityApps</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>u/GlitteringSuit5341</t>
         </is>
@@ -1970,10 +1964,10 @@
           <t>Anyone automated turning meeting notes into social media posts?</t>
         </is>
       </c>
-      <c r="I21" s="2" t="n">
+      <c r="I21" t="n">
         <v>45</v>
       </c>
-      <c r="J21" s="2" t="inlineStr">
+      <c r="J21" t="inlineStr">
         <is>
           <t>workflow_problem</t>
         </is>
@@ -1988,8 +1982,8 @@
           <t>One trick that cuts this down: flag the moment during the call instead of after. A quick note like 'post idea' with the timestamp means you're not rereading the whole summary later. Then the draft step is just 'turn this quote into a LinkedIn post in my voice', which any AI does fine. Keep the founder's exact words next to the draft so you don't accidentally change what they meant before you publish. n8n can handle the hand-off once the flagged notes land somewhere consistent.</t>
         </is>
       </c>
-      <c r="M21" s="2" t="inlineStr"/>
-      <c r="N21" s="2" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
       <c r="O21" s="2" t="inlineStr">
         <is>
           <t>Not read: Reddit returned 403 for subreddit rules from this environment</t>
@@ -1997,12 +1991,12 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="A22" t="inlineStr">
         <is>
           <t>2 engagement (discussion)</t>
         </is>
       </c>
-      <c r="B22" s="2" t="n">
+      <c r="B22" t="n">
         <v>21</v>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -2015,30 +2009,30 @@
           <t>https://www.reddit.com/r/Notion/comments/1wk288j/how_do_you_keep_a_shared_ai_meeting_notes/</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>post</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>r/Notion</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="G22" t="inlineStr">
         <is>
           <t>u/Antique-Anybody-1343</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr">
+      <c r="H22" t="inlineStr">
         <is>
           <t>How do you keep a shared AI Meeting Notes database clean?</t>
         </is>
       </c>
-      <c r="I22" s="2" t="n">
+      <c r="I22" t="n">
         <v>45</v>
       </c>
-      <c r="J22" s="2" t="inlineStr">
+      <c r="J22" t="inlineStr">
         <is>
           <t>workflow_problem</t>
         </is>
@@ -2053,8 +2047,8 @@
           <t>This drift is really common. What usually helps is cutting properties down to the three that drive views (internal or external, team, type) and setting them from the meeting title with a naming convention like 'EXT | Acme | Discovery'. A Notion automation or a small script can then parse the title into properties, which is more reliable than mapping invitees. Attendees are worth keeping as a plain text field for search rather than a relation you have to maintain. Anyone else found a cleaner way?</t>
         </is>
       </c>
-      <c r="M22" s="2" t="inlineStr"/>
-      <c r="N22" s="2" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
       <c r="O22" s="2" t="inlineStr">
         <is>
           <t>Not read: Reddit returned 403 for subreddit rules from this environment</t>
@@ -2062,12 +2056,12 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+      <c r="A23" t="inlineStr">
         <is>
           <t>2 engagement (discussion)</t>
         </is>
       </c>
-      <c r="B23" s="2" t="n">
+      <c r="B23" t="n">
         <v>22</v>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -2080,17 +2074,17 @@
           <t>https://www.reddit.com/r/productivity/comments/1witmm6/marketing_people_wearing_10_hats_what_have_you/</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>post</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>r/productivity</t>
         </is>
       </c>
-      <c r="G23" s="2" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>u/Vivi-vivi-S</t>
         </is>
@@ -2100,10 +2094,10 @@
           <t>Marketing people wearing 10 hats — what have you actually automated with AI?</t>
         </is>
       </c>
-      <c r="I23" s="2" t="n">
+      <c r="I23" t="n">
         <v>40</v>
       </c>
-      <c r="J23" s="2" t="inlineStr">
+      <c r="J23" t="inlineStr">
         <is>
           <t>workflow_problem</t>
         </is>
@@ -2118,8 +2112,8 @@
           <t>A common one that sticks is the meeting step: notes come out of the call already split into decisions, action items with owners and open questions, and only the action items get pushed into the task tool after a quick human check. The check matters; fully automatic task creation tends to turn 'we could' into fake tasks. Auto-generated reports are a common one people abandon, because they end up rewriting them anyway. Boring rule: automate the handoff, not the judgement.</t>
         </is>
       </c>
-      <c r="M23" s="2" t="inlineStr"/>
-      <c r="N23" s="2" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
       <c r="O23" s="2" t="inlineStr">
         <is>
           <t>Not read: Reddit returned 403 for subreddit rules from this environment</t>
@@ -2127,12 +2121,12 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="A24" t="inlineStr">
         <is>
           <t>2 engagement (discussion)</t>
         </is>
       </c>
-      <c r="B24" s="2" t="n">
+      <c r="B24" t="n">
         <v>23</v>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -2145,17 +2139,17 @@
           <t>https://www.reddit.com/r/HOA/comments/1wkn4pc/are_you_using_ai_to_take_your_meeting/</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>post</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t>r/HOA</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>u/soshinyapp</t>
         </is>
@@ -2165,15 +2159,15 @@
           <t>Are you using AI to take your meeting notes-minutes [ALL] [N/A]</t>
         </is>
       </c>
-      <c r="I24" s="2" t="n">
+      <c r="I24" t="n">
         <v>40</v>
       </c>
-      <c r="J24" s="2" t="inlineStr">
+      <c r="J24" t="inlineStr">
         <is>
           <t>general_discussion</t>
         </is>
       </c>
-      <c r="K24" s="2" t="inlineStr">
+      <c r="K24" t="inlineStr">
         <is>
           <t>HOA board minutes poll. Engagement only.</t>
         </is>
@@ -2183,8 +2177,8 @@
           <t>AI can be useful for the first draft of minutes, but minutes are a legal record, so the secretary still has to own them. What works: record with the board's consent, let the tool draft motions, votes and action items, then the secretary checks each motion and vote against the recording before the draft goes out for approval. Anything the tool summarises should be checkable against the moment it was said. Where it goes wrong is when the AI summary is approved as-is.</t>
         </is>
       </c>
-      <c r="M24" s="2" t="inlineStr"/>
-      <c r="N24" s="2" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
       <c r="O24" s="2" t="inlineStr">
         <is>
           <t>Not read: Reddit returned 403 for subreddit rules from this environment</t>
@@ -2192,12 +2186,12 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+      <c r="A25" t="inlineStr">
         <is>
           <t>2 engagement (discussion)</t>
         </is>
       </c>
-      <c r="B25" s="2" t="n">
+      <c r="B25" t="n">
         <v>24</v>
       </c>
       <c r="C25" s="3" t="inlineStr">
@@ -2210,30 +2204,30 @@
           <t>https://www.reddit.com/r/GenAiApps/comments/1wkxayl/id_like_meeting_apps_to_flag_tasks_with_no/</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>post</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>r/GenAiApps</t>
         </is>
       </c>
-      <c r="G25" s="2" t="inlineStr">
+      <c r="G25" t="inlineStr">
         <is>
           <t>u/lifeguard_8</t>
         </is>
       </c>
-      <c r="H25" s="2" t="inlineStr">
+      <c r="H25" t="inlineStr">
         <is>
           <t>I'd like meeting apps to flag tasks with no confirmed owner</t>
         </is>
       </c>
-      <c r="I25" s="2" t="n">
+      <c r="I25" t="n">
         <v>40</v>
       </c>
-      <c r="J25" s="2" t="inlineStr">
+      <c r="J25" t="inlineStr">
         <is>
           <t>workflow_problem</t>
         </is>
@@ -2248,8 +2242,8 @@
           <t>Agree, 'agreed but unowned' deserves its own section. A habit that works well in standups is ending with a 30-second owner check: read the action items out loud and anyone unassigned gets an owner or gets dropped. Tools help most when every action item links back to the moment it came from, so you can tell 'we should ask Sam' from 'Sam said yes'. Does Vomo keep the source moment next to each item?</t>
         </is>
       </c>
-      <c r="M25" s="2" t="inlineStr"/>
-      <c r="N25" s="2" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
       <c r="O25" s="2" t="inlineStr">
         <is>
           <t>Not read: Reddit returned 403 for subreddit rules from this environment</t>
@@ -2257,12 +2251,12 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="A26" t="inlineStr">
         <is>
           <t>2 engagement (discussion)</t>
         </is>
       </c>
-      <c r="B26" s="2" t="n">
+      <c r="B26" t="n">
         <v>25</v>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -2275,35 +2269,35 @@
           <t>https://www.reddit.com/r/projectmanagers/comments/1wuc4j7/aigenerated_project_updates_useful_or_just_more/</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>post</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="F26" t="inlineStr">
         <is>
           <t>r/projectmanagers</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G26" t="inlineStr">
         <is>
           <t>u/Kripa_HR</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="H26" t="inlineStr">
         <is>
           <t>AI-generated project updates: useful or just more noise?</t>
         </is>
       </c>
-      <c r="I26" s="2" t="n">
+      <c r="I26" t="n">
         <v>15</v>
       </c>
-      <c r="J26" s="2" t="inlineStr">
+      <c r="J26" t="inlineStr">
         <is>
           <t>general_discussion</t>
         </is>
       </c>
-      <c r="K26" s="2" t="inlineStr">
+      <c r="K26" t="inlineStr">
         <is>
           <t>PM discussion about AI status reports.</t>
         </is>
@@ -2313,8 +2307,8 @@
           <t>I'd trust the draft if every line traces back to a source: the ticket, the doc or the moment in the meeting where it was said. Without that, it's another report nobody believes. What a PM still has to own is the judgement: what's actually at risk, what changed since last week, and what needs a decision from someone. AI is good at collecting the facts, much less good at deciding which two of them matter.</t>
         </is>
       </c>
-      <c r="M26" s="2" t="inlineStr"/>
-      <c r="N26" s="2" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
       <c r="O26" s="2" t="inlineStr">
         <is>
           <t>Not read: Reddit returned 403 for subreddit rules from this environment</t>
@@ -2322,12 +2316,12 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+      <c r="A27" t="inlineStr">
         <is>
           <t>2 engagement (discussion)</t>
         </is>
       </c>
-      <c r="B27" s="2" t="n">
+      <c r="B27" t="n">
         <v>26</v>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -2340,17 +2334,17 @@
           <t>https://www.reddit.com/r/ProjectCoordinators/comments/1x0tcrp/70_of_project_orgs_now_use_ai_up_from_36_two/</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="E27" t="inlineStr">
         <is>
           <t>post</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr">
+      <c r="F27" t="inlineStr">
         <is>
           <t>r/ProjectCoordinators</t>
         </is>
       </c>
-      <c r="G27" s="2" t="inlineStr">
+      <c r="G27" t="inlineStr">
         <is>
           <t>u/Exciting_Tip3020</t>
         </is>
@@ -2360,10 +2354,10 @@
           <t>70% of project orgs now use AI (up from 36% two years ago), but what's actually earning its keep?</t>
         </is>
       </c>
-      <c r="I27" s="2" t="n">
+      <c r="I27" t="n">
         <v>20</v>
       </c>
-      <c r="J27" s="2" t="inlineStr">
+      <c r="J27" t="inlineStr">
         <is>
           <t>general_discussion</t>
         </is>
@@ -2381,10 +2375,10 @@
       <c r="M27" s="2" t="inlineStr">
         <is>
           <t>Meeting notes is the one that tends to stick, mostly because it removes the 'who's taking notes' problem and makes follow-ups faster. What makes it trustworthy is timestamps on every action item, so checking a disputed detail takes seconds. What people often drop: AI-written status reports, because they get rewritten every time. Risk brainstorming is decent as a checklist generator but not as a judgement call.
-I work on Lynkk, so I'm biased, but that's the setup it's built for: no-bot recording on Mac or Chrome, and a brief with decisions and action items that link back to the recording.</t>
-        </is>
-      </c>
-      <c r="N27" s="2" t="inlineStr">
+(Disclosure: I'm on the Lynkk team, which is a meeting notes tool, so weigh my vote accordingly.)</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
         <is>
           <t>If you want to try it, there's a free plan at lynkk.ai.</t>
         </is>
@@ -2396,12 +2390,12 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="A28" t="inlineStr">
         <is>
           <t>2 engagement (discussion)</t>
         </is>
       </c>
-      <c r="B28" s="2" t="n">
+      <c r="B28" t="n">
         <v>27</v>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -2414,17 +2408,17 @@
           <t>https://www.reddit.com/r/AIWritingLounge/comments/1wv37k6/do_you_use_ai_to_write_meeting_notes_or_do_you/</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="E28" t="inlineStr">
         <is>
           <t>post</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="F28" t="inlineStr">
         <is>
           <t>r/AIWritingLounge</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="G28" t="inlineStr">
         <is>
           <t>u/No-Tap-6768</t>
         </is>
@@ -2434,15 +2428,15 @@
           <t>Do you use AI to write meeting notes, or do you prefer summarizing them yourself?</t>
         </is>
       </c>
-      <c r="I28" s="2" t="n">
+      <c r="I28" t="n">
         <v>30</v>
       </c>
-      <c r="J28" s="2" t="inlineStr">
+      <c r="J28" t="inlineStr">
         <is>
           <t>general_discussion</t>
         </is>
       </c>
-      <c r="K28" s="2" t="inlineStr">
+      <c r="K28" t="inlineStr">
         <is>
           <t>Title-only poll. Short engagement reply.</t>
         </is>
@@ -2452,8 +2446,8 @@
           <t>Both works best. Let AI capture everything so you can pay attention in the meeting, then spend two minutes after the call checking the action items and decisions against the recording. Writing a few lines in your own words afterwards still helps you remember what matters. The AI part is the record, the summary in my head is the understanding.</t>
         </is>
       </c>
-      <c r="M28" s="2" t="inlineStr"/>
-      <c r="N28" s="2" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
       <c r="O28" s="2" t="inlineStr">
         <is>
           <t>Not read: Reddit returned 403 for subreddit rules from this environment</t>
@@ -2461,12 +2455,12 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+      <c r="A29" t="inlineStr">
         <is>
           <t>2 engagement (discussion)</t>
         </is>
       </c>
-      <c r="B29" s="2" t="n">
+      <c r="B29" t="n">
         <v>28</v>
       </c>
       <c r="C29" s="3" t="inlineStr">
@@ -2479,30 +2473,30 @@
           <t>https://www.reddit.com/r/PLAUDAI/comments/1x0n25s/plaud_ai_vs_claude_vs_gemini/</t>
         </is>
       </c>
-      <c r="E29" s="2" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>post</t>
         </is>
       </c>
-      <c r="F29" s="2" t="inlineStr">
+      <c r="F29" t="inlineStr">
         <is>
           <t>r/PLAUDAI</t>
         </is>
       </c>
-      <c r="G29" s="2" t="inlineStr">
+      <c r="G29" t="inlineStr">
         <is>
           <t>u/noodleJam-EU</t>
         </is>
       </c>
-      <c r="H29" s="2" t="inlineStr">
+      <c r="H29" t="inlineStr">
         <is>
           <t>Plaud Ai vs Claude vs Gemini</t>
         </is>
       </c>
-      <c r="I29" s="2" t="n">
+      <c r="I29" t="n">
         <v>30</v>
       </c>
-      <c r="J29" s="2" t="inlineStr">
+      <c r="J29" t="inlineStr">
         <is>
           <t>general_discussion</t>
         </is>
@@ -2517,8 +2511,8 @@
           <t>Interesting test. One thing I'd add: the gap between tools often shrinks a lot when the prompt asks for a fixed structure (decisions, action items with owner and date, open questions, risks) instead of a general summary, so it may be worth running Plaud's custom template with the same prompt you gave Claude. Speaker names matter too; 'Speaker 9' makes even a good summary hard to use. Did you check how each one handled things that were suggested but never agreed?</t>
         </is>
       </c>
-      <c r="M29" s="2" t="inlineStr"/>
-      <c r="N29" s="2" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr"/>
       <c r="O29" s="2" t="inlineStr">
         <is>
           <t>Not read: Reddit returned 403 for subreddit rules from this environment</t>
@@ -2526,12 +2520,12 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="A30" t="inlineStr">
         <is>
           <t>2 engagement (discussion)</t>
         </is>
       </c>
-      <c r="B30" s="2" t="n">
+      <c r="B30" t="n">
         <v>29</v>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -2544,35 +2538,35 @@
           <t>https://www.reddit.com/r/DoesAnybodyElse/comments/1wrvmal/dae_actually_have_an_easier_life_with_ai/</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="E30" t="inlineStr">
         <is>
           <t>post</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="F30" t="inlineStr">
         <is>
           <t>r/DoesAnybodyElse</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="G30" t="inlineStr">
         <is>
           <t>u/Parzival_b</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr">
+      <c r="H30" t="inlineStr">
         <is>
           <t>DAE actually have an easier life with AI?</t>
         </is>
       </c>
-      <c r="I30" s="2" t="n">
+      <c r="I30" t="n">
         <v>10</v>
       </c>
-      <c r="J30" s="2" t="inlineStr">
+      <c r="J30" t="inlineStr">
         <is>
           <t>general_discussion</t>
         </is>
       </c>
-      <c r="K30" s="2" t="inlineStr">
+      <c r="K30" t="inlineStr">
         <is>
           <t>General AI discussion. Light, friendly engagement.</t>
         </is>
@@ -2582,8 +2576,8 @@
           <t>Mixed is a fair description. The tools that tend to stick are the boring ones where checking is cheap: meeting notes you can verify against the recording, and drafts you'd have rewritten anyway. The ones people drop are where checking takes as long as doing it yourself. Fact-checking every output gets a lot easier when the tool shows you exactly where each claim came from.</t>
         </is>
       </c>
-      <c r="M30" s="2" t="inlineStr"/>
-      <c r="N30" s="2" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr"/>
       <c r="O30" s="2" t="inlineStr">
         <is>
           <t>Not read: Reddit returned 403 for subreddit rules from this environment</t>
@@ -2591,12 +2585,12 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr">
+      <c r="A31" t="inlineStr">
         <is>
           <t>2 engagement (discussion)</t>
         </is>
       </c>
-      <c r="B31" s="2" t="n">
+      <c r="B31" t="n">
         <v>30</v>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -2609,17 +2603,17 @@
           <t>https://www.reddit.com/r/AIWorkStack/comments/1wtsh32/how_i_use_ai_workflow_automation_to_save_time/</t>
         </is>
       </c>
-      <c r="E31" s="2" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>post</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr">
+      <c r="F31" t="inlineStr">
         <is>
           <t>r/AIWorkStack</t>
         </is>
       </c>
-      <c r="G31" s="2" t="inlineStr">
+      <c r="G31" t="inlineStr">
         <is>
           <t>u/lebron7</t>
         </is>
@@ -2629,10 +2623,10 @@
           <t>How I use AI workflow automation to save time without losing quality</t>
         </is>
       </c>
-      <c r="I31" s="2" t="n">
+      <c r="I31" t="n">
         <v>10</v>
       </c>
-      <c r="J31" s="2" t="inlineStr">
+      <c r="J31" t="inlineStr">
         <is>
           <t>general_discussion</t>
         </is>
@@ -2650,10 +2644,10 @@
       <c r="M31" s="2" t="inlineStr">
         <is>
           <t>Agree on keeping decisions manual. A big win for a lot of teams is the meeting step: recording calls, getting decisions and action items pulled out, and only then pushing the confirmed items into the task tool. The failure mode is automating task creation straight from the transcript, because suggestions turn into tasks nobody agreed to. A human check in the middle fixes it.
-I work on Lynkk, so I'm biased, but that's how we built the Jira step: it's a manual send from the note, not automatic.</t>
-        </is>
-      </c>
-      <c r="N31" s="2" t="inlineStr">
+(I work on Lynkk, and that's how its Jira step works: you send items by hand, nothing goes in automatically.)</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
         <is>
           <t>If you want to try it, there's a free plan at lynkk.ai.</t>
         </is>
@@ -2665,12 +2659,12 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="A32" t="inlineStr">
         <is>
           <t>2 engagement (discussion)</t>
         </is>
       </c>
-      <c r="B32" s="2" t="n">
+      <c r="B32" t="n">
         <v>31</v>
       </c>
       <c r="C32" s="3" t="inlineStr">
@@ -2683,17 +2677,17 @@
           <t>https://www.reddit.com/r/negotiation/comments/1x1qct6/is_there_an_ai_tool_that_can_tell_me_exactly/</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>comment</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="F32" t="inlineStr">
         <is>
           <t>r/negotiation</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="G32" t="inlineStr">
         <is>
           <t>u/belligerent_vogue</t>
         </is>
@@ -2703,10 +2697,10 @@
           <t>Is there an AI tool that can tell me exactly where a sales negotiation went wrong?</t>
         </is>
       </c>
-      <c r="I32" s="2" t="n">
+      <c r="I32" t="n">
         <v>40</v>
       </c>
-      <c r="J32" s="2" t="inlineStr">
+      <c r="J32" t="inlineStr">
         <is>
           <t>problem_seeking_solution</t>
         </is>
@@ -2721,8 +2715,8 @@
           <t>For phone calls, check two things before any demo: whether the tool can record your actual phone setup (softphone or dialer) with both sides on separate channels, and whether you can jump to a moment and leave a timestamped comment for the rep. Then test it on five lost deals and see if it finds the turn you'd have found yourself. If it can't find the moment the tone shifted on calls you already know well, it won't on new ones.</t>
         </is>
       </c>
-      <c r="M32" s="2" t="inlineStr"/>
-      <c r="N32" s="2" t="inlineStr"/>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="inlineStr"/>
       <c r="O32" s="2" t="inlineStr">
         <is>
           <t>Not read: Reddit returned 403 for subreddit rules from this environment</t>
@@ -2730,12 +2724,12 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
+      <c r="A33" t="inlineStr">
         <is>
           <t>2 engagement (discussion)</t>
         </is>
       </c>
-      <c r="B33" s="2" t="n">
+      <c r="B33" t="n">
         <v>32</v>
       </c>
       <c r="C33" s="3" t="inlineStr">
@@ -2748,30 +2742,30 @@
           <t>https://www.reddit.com/r/PlaudNoteUsers/comments/1x12i9y/what_ai_note_taking_apps_are_you_using_for/</t>
         </is>
       </c>
-      <c r="E33" s="2" t="inlineStr">
+      <c r="E33" t="inlineStr">
         <is>
           <t>comment</t>
         </is>
       </c>
-      <c r="F33" s="2" t="inlineStr">
+      <c r="F33" t="inlineStr">
         <is>
           <t>r/PlaudNoteUsers</t>
         </is>
       </c>
-      <c r="G33" s="2" t="inlineStr">
+      <c r="G33" t="inlineStr">
         <is>
           <t>u/QuietlyKevin07</t>
         </is>
       </c>
-      <c r="H33" s="2" t="inlineStr">
+      <c r="H33" t="inlineStr">
         <is>
           <t>What AI note taking apps are you using for meetings?</t>
         </is>
       </c>
-      <c r="I33" s="2" t="n">
+      <c r="I33" t="n">
         <v>35</v>
       </c>
-      <c r="J33" s="2" t="inlineStr">
+      <c r="J33" t="inlineStr">
         <is>
           <t>comparison</t>
         </is>
@@ -2789,10 +2783,10 @@
       <c r="M33" s="2" t="inlineStr">
         <is>
           <t>Long meetings are where most note takers get vague: the summary covers the first half well and compresses the rest. Two things help: a tool that splits the brief into topics with timestamps, and checking a 90-minute real meeting rather than a 20-minute demo before you decide.
-I work on Lynkk, so I'm biased: its brief has takeaways with timestamps that play the recording from that moment, and each recording can run up to 2 hours.</t>
-        </is>
-      </c>
-      <c r="N33" s="2" t="inlineStr">
+(Disclosure: I work on Lynkk. Its notes have timestamps you can click to replay, and a recording can run up to 2 hours.)</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
         <is>
           <t>If you want to try it, there's a free plan at lynkk.ai.</t>
         </is>
@@ -2804,12 +2798,12 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="A34" t="inlineStr">
         <is>
           <t>2 engagement (discussion)</t>
         </is>
       </c>
-      <c r="B34" s="2" t="n">
+      <c r="B34" t="n">
         <v>33</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -2822,17 +2816,17 @@
           <t>https://www.reddit.com/r/LocalLLM/comments/1x2918k/hardware_and_llm_choice_for_business_ops_project/</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t>post</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="F34" t="inlineStr">
         <is>
           <t>r/LocalLLM</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="G34" t="inlineStr">
         <is>
           <t>u/Hefty-Divide7339</t>
         </is>
@@ -2842,10 +2836,10 @@
           <t>Hardware and LLM choice for business ops / project management</t>
         </is>
       </c>
-      <c r="I34" s="2" t="n">
+      <c r="I34" t="n">
         <v>35</v>
       </c>
-      <c r="J34" s="2" t="inlineStr">
+      <c r="J34" t="inlineStr">
         <is>
           <t>problem_seeking_solution</t>
         </is>
@@ -2860,8 +2854,8 @@
           <t>For minutes from recordings, the model size matters less than the pipeline: a good local transcription model with speaker labels, then a fixed minutes template (attendees, decisions, actions with owner and date, open points) fed to the LLM. A mid-size model handles that well; the big models earn their keep on the contract analysis side. I'd benchmark with one real meeting rather than fake contracts, since speaker attribution is usually where it breaks.</t>
         </is>
       </c>
-      <c r="M34" s="2" t="inlineStr"/>
-      <c r="N34" s="2" t="inlineStr"/>
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" t="inlineStr"/>
       <c r="O34" s="2" t="inlineStr">
         <is>
           <t>Not read: Reddit returned 403 for subreddit rules from this environment</t>
@@ -2869,12 +2863,12 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+      <c r="A35" t="inlineStr">
         <is>
           <t>2 engagement (discussion)</t>
         </is>
       </c>
-      <c r="B35" s="2" t="n">
+      <c r="B35" t="n">
         <v>34</v>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -2887,17 +2881,17 @@
           <t>https://www.reddit.com/r/LocalLLaMA/comments/1wwnpxj/anyone_using_a_local_ai_meeting_notes_setup/</t>
         </is>
       </c>
-      <c r="E35" s="2" t="inlineStr">
+      <c r="E35" t="inlineStr">
         <is>
           <t>post</t>
         </is>
       </c>
-      <c r="F35" s="2" t="inlineStr">
+      <c r="F35" t="inlineStr">
         <is>
           <t>r/LocalLLaMA</t>
         </is>
       </c>
-      <c r="G35" s="2" t="inlineStr">
+      <c r="G35" t="inlineStr">
         <is>
           <t>u/Sash17</t>
         </is>
@@ -2907,15 +2901,15 @@
           <t>Anyone using a local AI meeting notes setup instead of Fathom?</t>
         </is>
       </c>
-      <c r="I35" s="2" t="n">
+      <c r="I35" t="n">
         <v>30</v>
       </c>
-      <c r="J35" s="2" t="inlineStr">
+      <c r="J35" t="inlineStr">
         <is>
           <t>tool_recommendation</t>
         </is>
       </c>
-      <c r="K35" s="2" t="inlineStr">
+      <c r="K35" t="inlineStr">
         <is>
           <t>Wants a local setup. Engage only; no product.</t>
         </is>
@@ -2925,8 +2919,8 @@
           <t>Whisper plus a local LLM works, but the parts that take effort are speaker labels and search. Record your mic and the system audio on separate channels so 'you' and 'others' are clean, run diarization only on the others channel, and store transcripts as plain files with the summary on top so search stays simple. The summary prompt matters more than the model: a fixed structure of decisions, actions and open questions beats 'summarize this'.</t>
         </is>
       </c>
-      <c r="M35" s="2" t="inlineStr"/>
-      <c r="N35" s="2" t="inlineStr"/>
+      <c r="M35" t="inlineStr"/>
+      <c r="N35" t="inlineStr"/>
       <c r="O35" s="2" t="inlineStr">
         <is>
           <t>Not read: Reddit returned 403 for subreddit rules from this environment</t>
@@ -2934,12 +2928,12 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="A36" t="inlineStr">
         <is>
           <t>2 engagement (discussion)</t>
         </is>
       </c>
-      <c r="B36" s="2" t="n">
+      <c r="B36" t="n">
         <v>35</v>
       </c>
       <c r="C36" s="3" t="inlineStr">
@@ -2952,17 +2946,17 @@
           <t>https://www.reddit.com/r/PLAUDAI/comments/1x1tha4/lawyers_using_plaud_or_other_ai_notetakers_for/</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="E36" t="inlineStr">
         <is>
           <t>comment</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="F36" t="inlineStr">
         <is>
           <t>r/PLAUDAI</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="G36" t="inlineStr">
         <is>
           <t>u/lookamazed</t>
         </is>
@@ -2972,10 +2966,10 @@
           <t>Lawyers using Plaud or other AI note-takers for client consultations — what has your experience been?</t>
         </is>
       </c>
-      <c r="I36" s="2" t="n">
+      <c r="I36" t="n">
         <v>25</v>
       </c>
-      <c r="J36" s="2" t="inlineStr">
+      <c r="J36" t="inlineStr">
         <is>
           <t>general_discussion</t>
         </is>
@@ -2990,8 +2984,8 @@
           <t>Verbosity usually improves more from limits than from longer templates: cap each section (5 decisions, 5 actions, 3 open questions), ask for owner and date on every action, and tell it to leave out anything not explicitly agreed. Asking for a quote or timestamp next to each decision also cuts the padding, because the model can't pad what it has to cite.</t>
         </is>
       </c>
-      <c r="M36" s="2" t="inlineStr"/>
-      <c r="N36" s="2" t="inlineStr"/>
+      <c r="M36" t="inlineStr"/>
+      <c r="N36" t="inlineStr"/>
       <c r="O36" s="2" t="inlineStr">
         <is>
           <t>Not read: Reddit returned 403 for subreddit rules from this environment</t>
@@ -2999,12 +2993,12 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr">
+      <c r="A37" t="inlineStr">
         <is>
           <t>2 engagement (discussion)</t>
         </is>
       </c>
-      <c r="B37" s="2" t="n">
+      <c r="B37" t="n">
         <v>36</v>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -3017,17 +3011,17 @@
           <t>https://www.reddit.com/r/AIVoice_Agents/comments/1x1quo3/is_anyone_using_ai_voice_tools_to_help_support/</t>
         </is>
       </c>
-      <c r="E37" s="2" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>post</t>
         </is>
       </c>
-      <c r="F37" s="2" t="inlineStr">
+      <c r="F37" t="inlineStr">
         <is>
           <t>r/AIVoice_Agents</t>
         </is>
       </c>
-      <c r="G37" s="2" t="inlineStr">
+      <c r="G37" t="inlineStr">
         <is>
           <t>u/scandalous_mohamed</t>
         </is>
@@ -3037,10 +3031,10 @@
           <t>Is anyone using AI voice tools to help support agents during calls instead of replacing them?</t>
         </is>
       </c>
-      <c r="I37" s="2" t="n">
+      <c r="I37" t="n">
         <v>25</v>
       </c>
-      <c r="J37" s="2" t="inlineStr">
+      <c r="J37" t="inlineStr">
         <is>
           <t>problem_seeking_solution</t>
         </is>
@@ -3055,8 +3049,8 @@
           <t>The call notes part is usually the easiest win: automatic summaries with the customer's issue, what was promised and next steps cut after-call work a lot. Real-time suggestions are harder; they're only useful if the knowledge base is clean, otherwise reps learn to ignore them within a week. I'd pilot notes first, then add live prompts for the two or three call types that cause most holds.</t>
         </is>
       </c>
-      <c r="M37" s="2" t="inlineStr"/>
-      <c r="N37" s="2" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" t="inlineStr"/>
       <c r="O37" s="2" t="inlineStr">
         <is>
           <t>Not read: Reddit returned 403 for subreddit rules from this environment</t>
@@ -3064,12 +3058,12 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="A38" t="inlineStr">
         <is>
           <t>2 engagement (discussion)</t>
         </is>
       </c>
-      <c r="B38" s="2" t="n">
+      <c r="B38" t="n">
         <v>37</v>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -3082,30 +3076,30 @@
           <t>https://www.reddit.com/r/PMCareers/comments/1wiznmp/is_it_my_pm_skills_or_this_org_is_an_absolute_mess/</t>
         </is>
       </c>
-      <c r="E38" s="2" t="inlineStr">
+      <c r="E38" t="inlineStr">
         <is>
           <t>post</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="F38" t="inlineStr">
         <is>
           <t>r/PMCareers</t>
         </is>
       </c>
-      <c r="G38" s="2" t="inlineStr">
+      <c r="G38" t="inlineStr">
         <is>
           <t>u/Sad_Impress4747</t>
         </is>
       </c>
-      <c r="H38" s="2" t="inlineStr">
+      <c r="H38" t="inlineStr">
         <is>
           <t>Is it my PM skills or this org is an absolute mess?</t>
         </is>
       </c>
-      <c r="I38" s="2" t="n">
+      <c r="I38" t="n">
         <v>20</v>
       </c>
-      <c r="J38" s="2" t="inlineStr">
+      <c r="J38" t="inlineStr">
         <is>
           <t>workflow_problem</t>
         </is>
@@ -3120,8 +3114,8 @@
           <t>Taking notes and chasing dependencies is normal early in a PMO, but owning 40 to 70 projects with no context is not. One practical tip: send the report within an hour, with three headings (decisions, actions with owner and date, open questions) and ask attendees to correct it by end of day. It turns note-taking into the record people rely on, which is how you start getting pulled in earlier.</t>
         </is>
       </c>
-      <c r="M38" s="2" t="inlineStr"/>
-      <c r="N38" s="2" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="inlineStr"/>
       <c r="O38" s="2" t="inlineStr">
         <is>
           <t>Not read: Reddit returned 403 for subreddit rules from this environment</t>
@@ -3129,12 +3123,12 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr">
+      <c r="A39" t="inlineStr">
         <is>
           <t>2 engagement (discussion)</t>
         </is>
       </c>
-      <c r="B39" s="2" t="n">
+      <c r="B39" t="n">
         <v>38</v>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -3147,17 +3141,17 @@
           <t>https://www.reddit.com/r/ChatGPT/comments/1wm4p5t/why_does_ai_sometimes_make_my_summary_longer_than/</t>
         </is>
       </c>
-      <c r="E39" s="2" t="inlineStr">
+      <c r="E39" t="inlineStr">
         <is>
           <t>post</t>
         </is>
       </c>
-      <c r="F39" s="2" t="inlineStr">
+      <c r="F39" t="inlineStr">
         <is>
           <t>r/ChatGPT</t>
         </is>
       </c>
-      <c r="G39" s="2" t="inlineStr">
+      <c r="G39" t="inlineStr">
         <is>
           <t>u/yi111</t>
         </is>
@@ -3167,15 +3161,15 @@
           <t>Why does AI sometimes make my “summary” longer than the thing I wanted summarized?</t>
         </is>
       </c>
-      <c r="I39" s="2" t="n">
+      <c r="I39" t="n">
         <v>10</v>
       </c>
-      <c r="J39" s="2" t="inlineStr">
+      <c r="J39" t="inlineStr">
         <is>
           <t>general_discussion</t>
         </is>
       </c>
-      <c r="K39" s="2" t="inlineStr">
+      <c r="K39" t="inlineStr">
         <is>
           <t>ChatGPT summary length discussion. Light engagement.</t>
         </is>
@@ -3185,8 +3179,8 @@
           <t>Ruthless cut, usually. What works is giving it a shape instead of a length: 'three decisions, three actions with owners, anything unresolved, nothing else'. Completeness creeps back in when the prompt is open-ended. For meetings specifically, separating what was agreed from what was only discussed cuts the length more than any word limit.</t>
         </is>
       </c>
-      <c r="M39" s="2" t="inlineStr"/>
-      <c r="N39" s="2" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" t="inlineStr"/>
       <c r="O39" s="2" t="inlineStr">
         <is>
           <t>Not read: Reddit returned 403 for subreddit rules from this environment</t>

</xml_diff>